<commit_message>
refactor: adjusting report excel template
</commit_message>
<xml_diff>
--- a/resources/excel/template_report_inspeksi.xlsx
+++ b/resources/excel/template_report_inspeksi.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\qhs-dashboard-ubs-gold\resources\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BAE1FD7-5886-448C-9BA1-0049596DBC18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED48B134-327E-4DA7-917B-579E00C104F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{64A5FF42-60C1-45C5-A4B5-115E774A40CA}"/>
+    <workbookView xWindow="4530" yWindow="3960" windowWidth="21600" windowHeight="11835" xr2:uid="{64A5FF42-60C1-45C5-A4B5-115E774A40CA}"/>
   </bookViews>
   <sheets>
     <sheet name="report" sheetId="3" r:id="rId1"/>
@@ -34,34 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="27">
-  <si>
-    <t>QHS Assisten Officer</t>
-  </si>
-  <si>
-    <t>Ass Man QMS</t>
-  </si>
-  <si>
-    <t>Temuan Open</t>
-  </si>
-  <si>
-    <t>Javiero Isroj W</t>
-  </si>
-  <si>
-    <t>Yanata Candra</t>
-  </si>
-  <si>
-    <t>Temuan Closed</t>
-  </si>
-  <si>
-    <t>Total temuan Mutu</t>
-  </si>
-  <si>
-    <t>Disetujui</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total temuan K3 </t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="15">
   <si>
     <t>(%)</t>
   </si>
@@ -99,15 +72,6 @@
     <t xml:space="preserve">: </t>
   </si>
   <si>
-    <t>Surabaya, …..</t>
-  </si>
-  <si>
-    <t>Dibuat &amp; Diperiksa</t>
-  </si>
-  <si>
-    <t>-</t>
-  </si>
-  <si>
     <t>Sistem Manajemen Terintegrasi (Mutu &amp; K3)</t>
   </si>
   <si>
@@ -121,7 +85,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -144,22 +108,11 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="8"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
     </font>
@@ -197,40 +150,12 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="9">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -246,60 +171,9 @@
       <left style="thin">
         <color rgb="FF000000"/>
       </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
@@ -344,24 +218,26 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
       <top style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left/>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
       <right style="thin">
-        <color indexed="64"/>
+        <color rgb="FF000000"/>
       </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
+      <top/>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
@@ -375,9 +251,11 @@
         <color rgb="FF000000"/>
       </right>
       <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
         <color indexed="64"/>
-      </top>
-      <bottom/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -385,74 +263,48 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="5" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -836,255 +688,254 @@
     <col min="3" max="3" width="22.28515625" style="1" customWidth="1"/>
     <col min="4" max="11" width="6.5703125" style="1" customWidth="1"/>
     <col min="12" max="12" width="11.7109375" style="1" customWidth="1"/>
-    <col min="13" max="13" width="13.5703125" style="1" customWidth="1"/>
+    <col min="13" max="13" width="15" style="1" customWidth="1"/>
     <col min="14" max="26" width="8.7109375" style="1" customWidth="1"/>
     <col min="27" max="16384" width="14.42578125" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="15" customHeight="1">
-      <c r="A1" s="30"/>
-      <c r="B1" s="33" t="s">
-        <v>26</v>
+      <c r="A1" s="4"/>
+      <c r="B1" s="13" t="s">
+        <v>14</v>
       </c>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
-      <c r="G1" s="33"/>
-      <c r="H1" s="33"/>
-      <c r="I1" s="33"/>
-      <c r="J1" s="33"/>
-      <c r="K1" s="35"/>
-      <c r="L1" s="30"/>
-      <c r="M1" s="36"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+      <c r="I1" s="13"/>
+      <c r="J1" s="13"/>
+      <c r="K1" s="6"/>
+      <c r="L1" s="4"/>
+      <c r="M1" s="11"/>
     </row>
     <row r="2" spans="1:13" ht="15" customHeight="1">
-      <c r="A2" s="30"/>
-      <c r="B2" s="33"/>
-      <c r="C2" s="33"/>
-      <c r="D2" s="33"/>
-      <c r="E2" s="33"/>
-      <c r="F2" s="33"/>
-      <c r="G2" s="33"/>
-      <c r="H2" s="33"/>
-      <c r="I2" s="33"/>
-      <c r="J2" s="33"/>
-      <c r="K2" s="35"/>
-      <c r="L2" s="30"/>
-      <c r="M2" s="36"/>
+      <c r="A2" s="4"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
+      <c r="H2" s="13"/>
+      <c r="I2" s="13"/>
+      <c r="J2" s="13"/>
+      <c r="K2" s="6"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="11"/>
     </row>
     <row r="3" spans="1:13" ht="21" customHeight="1">
-      <c r="A3" s="31"/>
-      <c r="B3" s="34" t="s">
-        <v>24</v>
+      <c r="B3" s="12" t="s">
+        <v>12</v>
       </c>
-      <c r="C3" s="34"/>
-      <c r="D3" s="34"/>
-      <c r="E3" s="34"/>
-      <c r="F3" s="34"/>
-      <c r="G3" s="34"/>
-      <c r="H3" s="34"/>
-      <c r="I3" s="34"/>
-      <c r="J3" s="34"/>
-      <c r="K3" s="29" t="s">
-        <v>25</v>
+      <c r="C3" s="12"/>
+      <c r="D3" s="12"/>
+      <c r="E3" s="12"/>
+      <c r="F3" s="12"/>
+      <c r="G3" s="12"/>
+      <c r="H3" s="12"/>
+      <c r="I3" s="12"/>
+      <c r="J3" s="12"/>
+      <c r="K3" s="3" t="s">
+        <v>13</v>
       </c>
-      <c r="M3" s="29" t="s">
-        <v>20</v>
+      <c r="M3" s="3" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:13">
-      <c r="A4" s="32" t="s">
-        <v>19</v>
+      <c r="A4" s="5" t="s">
+        <v>10</v>
       </c>
-      <c r="B4" s="23" t="s">
-        <v>18</v>
+      <c r="B4" s="2" t="s">
+        <v>9</v>
       </c>
-      <c r="C4" s="23" t="s">
-        <v>17</v>
+      <c r="C4" s="2" t="s">
+        <v>8</v>
       </c>
-      <c r="D4" s="22" t="s">
-        <v>16</v>
+      <c r="D4" s="14" t="s">
+        <v>7</v>
       </c>
-      <c r="E4" s="21"/>
-      <c r="F4" s="21"/>
-      <c r="G4" s="20"/>
-      <c r="H4" s="22" t="s">
-        <v>15</v>
+      <c r="E4" s="15"/>
+      <c r="F4" s="15"/>
+      <c r="G4" s="16"/>
+      <c r="H4" s="14" t="s">
+        <v>6</v>
       </c>
-      <c r="I4" s="21"/>
-      <c r="J4" s="21"/>
-      <c r="K4" s="20"/>
-      <c r="L4" s="19" t="s">
-        <v>14</v>
+      <c r="I4" s="15"/>
+      <c r="J4" s="15"/>
+      <c r="K4" s="16"/>
+      <c r="L4" s="17" t="s">
+        <v>5</v>
       </c>
-      <c r="M4" s="19" t="s">
-        <v>13</v>
+      <c r="M4" s="17" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="18"/>
       <c r="B5" s="18"/>
       <c r="C5" s="18"/>
-      <c r="D5" s="17" t="s">
-        <v>12</v>
+      <c r="D5" s="19" t="s">
+        <v>3</v>
       </c>
-      <c r="E5" s="17" t="s">
-        <v>11</v>
+      <c r="E5" s="19" t="s">
+        <v>2</v>
       </c>
-      <c r="F5" s="17" t="s">
-        <v>10</v>
+      <c r="F5" s="19" t="s">
+        <v>1</v>
       </c>
-      <c r="G5" s="17" t="s">
-        <v>9</v>
+      <c r="G5" s="19" t="s">
+        <v>0</v>
       </c>
-      <c r="H5" s="17" t="s">
-        <v>12</v>
+      <c r="H5" s="19" t="s">
+        <v>3</v>
       </c>
-      <c r="I5" s="17" t="s">
-        <v>11</v>
+      <c r="I5" s="19" t="s">
+        <v>2</v>
       </c>
-      <c r="J5" s="17" t="s">
-        <v>10</v>
+      <c r="J5" s="19" t="s">
+        <v>1</v>
       </c>
-      <c r="K5" s="17" t="s">
-        <v>9</v>
+      <c r="K5" s="19" t="s">
+        <v>0</v>
       </c>
-      <c r="L5" s="3"/>
-      <c r="M5" s="3"/>
+      <c r="L5" s="20"/>
+      <c r="M5" s="20"/>
     </row>
     <row r="6" spans="1:13">
-      <c r="A6" s="24">
-        <v>1</v>
-      </c>
-      <c r="B6" s="25" t="s">
-        <v>23</v>
-      </c>
-      <c r="C6" s="24" t="s">
-        <v>23</v>
-      </c>
-      <c r="D6" s="26" t="s">
-        <v>23</v>
-      </c>
-      <c r="E6" s="26" t="s">
-        <v>23</v>
-      </c>
-      <c r="F6" s="26" t="s">
-        <v>23</v>
-      </c>
-      <c r="G6" s="27">
-        <v>0</v>
-      </c>
-      <c r="H6" s="26" t="s">
-        <v>23</v>
-      </c>
-      <c r="I6" s="26" t="s">
-        <v>23</v>
-      </c>
-      <c r="J6" s="26" t="s">
-        <v>23</v>
-      </c>
-      <c r="K6" s="27">
-        <v>0</v>
-      </c>
-      <c r="L6" s="25" t="s">
-        <v>23</v>
-      </c>
-      <c r="M6" s="28">
-        <v>0</v>
-      </c>
+      <c r="B6" s="8"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
+      <c r="G6" s="10"/>
+      <c r="H6" s="9"/>
+      <c r="I6" s="9"/>
+      <c r="J6" s="9"/>
+      <c r="K6" s="10"/>
+      <c r="L6" s="8"/>
+      <c r="M6" s="10"/>
     </row>
-    <row r="8" spans="1:13">
-      <c r="A8" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8" s="12"/>
-      <c r="C8" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="D8" s="11">
-        <v>0</v>
-      </c>
-      <c r="L8" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="M8" s="15"/>
+    <row r="8" spans="1:13" ht="15" customHeight="1">
+      <c r="A8" s="7"/>
+      <c r="B8" s="7"/>
+      <c r="C8" s="7"/>
+      <c r="D8" s="7"/>
+      <c r="E8" s="7"/>
+      <c r="F8" s="7"/>
+      <c r="G8" s="7"/>
+      <c r="H8" s="7"/>
+      <c r="I8" s="7"/>
+      <c r="J8" s="7"/>
+      <c r="K8" s="7"/>
+      <c r="L8" s="7"/>
+      <c r="M8" s="7"/>
     </row>
     <row r="9" spans="1:13">
-      <c r="A9" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="B9" s="8"/>
-      <c r="C9" s="8" t="s">
-        <v>20</v>
-      </c>
+      <c r="A9" s="7"/>
+      <c r="B9" s="7"/>
+      <c r="C9" s="7"/>
       <c r="D9" s="7"/>
+      <c r="E9" s="7"/>
+      <c r="F9" s="7"/>
+      <c r="G9" s="7"/>
+      <c r="H9" s="7"/>
+      <c r="I9" s="7"/>
+      <c r="J9" s="7"/>
+      <c r="K9" s="7"/>
+      <c r="L9" s="7"/>
+      <c r="M9" s="7"/>
     </row>
     <row r="10" spans="1:13">
-      <c r="A10" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="B10" s="4"/>
-      <c r="C10" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="D10" s="3"/>
-      <c r="L10" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="M10" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="A10" s="7"/>
+      <c r="B10" s="7"/>
+      <c r="C10" s="7"/>
+      <c r="D10" s="7"/>
+      <c r="E10" s="7"/>
+      <c r="F10" s="7"/>
+      <c r="G10" s="7"/>
+      <c r="H10" s="7"/>
+      <c r="I10" s="7"/>
+      <c r="J10" s="7"/>
+      <c r="K10" s="7"/>
+      <c r="L10" s="7"/>
+      <c r="M10" s="7"/>
     </row>
     <row r="11" spans="1:13">
-      <c r="L11" s="14"/>
-      <c r="M11" s="14"/>
+      <c r="A11" s="7"/>
+      <c r="B11" s="7"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="7"/>
+      <c r="G11" s="7"/>
+      <c r="H11" s="7"/>
+      <c r="I11" s="7"/>
+      <c r="J11" s="7"/>
+      <c r="K11" s="7"/>
+      <c r="L11" s="7"/>
+      <c r="M11" s="7"/>
     </row>
-    <row r="12" spans="1:13">
-      <c r="A12" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="B12" s="12"/>
-      <c r="C12" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="D12" s="11">
-        <v>0</v>
-      </c>
-      <c r="L12" s="10"/>
-      <c r="M12" s="10"/>
+    <row r="12" spans="1:13" ht="15" customHeight="1">
+      <c r="A12" s="7"/>
+      <c r="B12" s="7"/>
+      <c r="C12" s="7"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="7"/>
+      <c r="F12" s="7"/>
+      <c r="G12" s="7"/>
+      <c r="H12" s="7"/>
+      <c r="I12" s="7"/>
+      <c r="J12" s="7"/>
+      <c r="K12" s="7"/>
+      <c r="L12" s="7"/>
+      <c r="M12" s="7"/>
     </row>
     <row r="13" spans="1:13">
-      <c r="A13" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="B13" s="8"/>
-      <c r="C13" s="8" t="s">
-        <v>20</v>
-      </c>
+      <c r="A13" s="7"/>
+      <c r="B13" s="7"/>
+      <c r="C13" s="7"/>
       <c r="D13" s="7"/>
-      <c r="L13" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="M13" s="6" t="s">
-        <v>3</v>
-      </c>
+      <c r="E13" s="7"/>
+      <c r="F13" s="7"/>
+      <c r="G13" s="7"/>
+      <c r="H13" s="7"/>
+      <c r="I13" s="7"/>
+      <c r="J13" s="7"/>
+      <c r="K13" s="7"/>
+      <c r="L13" s="7"/>
+      <c r="M13" s="7"/>
     </row>
     <row r="14" spans="1:13">
-      <c r="A14" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="B14" s="4"/>
-      <c r="C14" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="D14" s="3"/>
-      <c r="L14" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="M14" s="2" t="s">
-        <v>0</v>
-      </c>
+      <c r="A14" s="7"/>
+      <c r="B14" s="7"/>
+      <c r="C14" s="7"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="7"/>
+      <c r="G14" s="7"/>
+      <c r="H14" s="7"/>
+      <c r="I14" s="7"/>
+      <c r="J14" s="7"/>
+      <c r="K14" s="7"/>
+      <c r="L14" s="7"/>
+      <c r="M14" s="7"/>
+    </row>
+    <row r="15" spans="1:13" ht="15" customHeight="1">
+      <c r="A15" s="7"/>
+      <c r="B15" s="7"/>
+      <c r="C15" s="7"/>
+      <c r="D15" s="7"/>
+      <c r="E15" s="7"/>
+      <c r="F15" s="7"/>
+      <c r="G15" s="7"/>
+      <c r="H15" s="7"/>
+      <c r="I15" s="7"/>
+      <c r="J15" s="7"/>
+      <c r="K15" s="7"/>
+      <c r="L15" s="7"/>
+      <c r="M15" s="7"/>
     </row>
     <row r="18" ht="15.75" customHeight="1"/>
     <row r="19" ht="15.75" customHeight="1"/>
@@ -2067,17 +1918,14 @@
     <row r="996" ht="15.75" customHeight="1"/>
     <row r="997" ht="15.75" customHeight="1"/>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="7">
     <mergeCell ref="M1:M2"/>
-    <mergeCell ref="D12:D14"/>
     <mergeCell ref="B3:J3"/>
     <mergeCell ref="B1:J2"/>
     <mergeCell ref="D4:G4"/>
     <mergeCell ref="H4:K4"/>
     <mergeCell ref="L4:L5"/>
     <mergeCell ref="M4:M5"/>
-    <mergeCell ref="D8:D10"/>
-    <mergeCell ref="L8:M8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>

</xml_diff>